<commit_message>
Deploying to gh-pages from @ codeforIATI/codelists@56214b660bf2557f2d99cb7c193581a1aef67d30 🚀
</commit_message>
<xml_diff>
--- a/api/1/clv1/codelist/GLIDENumber.xlsx
+++ b/api/1/clv1/codelist/GLIDENumber.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17047" uniqueCount="8528">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17089" uniqueCount="8549">
   <si>
     <t>code</t>
   </si>
@@ -41,6 +41,69 @@
   </si>
   <si>
     <t>en</t>
+  </si>
+  <si>
+    <t>LS-2025-000165-MYS</t>
+  </si>
+  <si>
+    <t>EQ-2025-000164-IND</t>
+  </si>
+  <si>
+    <t>WF-2025-000163-BOL</t>
+  </si>
+  <si>
+    <t>EQ-2025-000162-RUS</t>
+  </si>
+  <si>
+    <t>FL-2025-000161-IDN</t>
+  </si>
+  <si>
+    <t>TC-2025-000160-CHN</t>
+  </si>
+  <si>
+    <t>EQ-2025-000159-AFG</t>
+  </si>
+  <si>
+    <t>FL-2025-000158-SSD</t>
+  </si>
+  <si>
+    <t>EP-2025-000157-COD</t>
+  </si>
+  <si>
+    <t>EQ-2025-000156-AFG</t>
+  </si>
+  <si>
+    <t>FR-2025-000155-KAZ</t>
+  </si>
+  <si>
+    <t>FL-2025-000154-SDN</t>
+  </si>
+  <si>
+    <t>EQ-2025-000153-AFG</t>
+  </si>
+  <si>
+    <t>DR-2025-000152-SYR</t>
+  </si>
+  <si>
+    <t>FL-2025-000151-YEM</t>
+  </si>
+  <si>
+    <t>FL-2025-000150-GIN</t>
+  </si>
+  <si>
+    <t>EP-2025-000149-TCD</t>
+  </si>
+  <si>
+    <t>DR-2025-000148-ETH</t>
+  </si>
+  <si>
+    <t>FL-2025-000147-CPV</t>
+  </si>
+  <si>
+    <t>FL-2025-000146-CPV</t>
+  </si>
+  <si>
+    <t>FL-2025-000145-GNQ</t>
   </si>
   <si>
     <t>TC-2025-000144-VNM</t>
@@ -25929,7 +25992,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G8521"/>
+  <dimension ref="A1:G8542"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -94115,6 +94178,174 @@
         <v>8</v>
       </c>
     </row>
+    <row r="8522" spans="1:4">
+      <c r="A8522" t="s">
+        <v>8528</v>
+      </c>
+      <c r="D8522" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8523" spans="1:4">
+      <c r="A8523" t="s">
+        <v>8529</v>
+      </c>
+      <c r="D8523" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8524" spans="1:4">
+      <c r="A8524" t="s">
+        <v>8530</v>
+      </c>
+      <c r="D8524" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8525" spans="1:4">
+      <c r="A8525" t="s">
+        <v>8531</v>
+      </c>
+      <c r="D8525" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8526" spans="1:4">
+      <c r="A8526" t="s">
+        <v>8532</v>
+      </c>
+      <c r="D8526" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8527" spans="1:4">
+      <c r="A8527" t="s">
+        <v>8533</v>
+      </c>
+      <c r="D8527" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8528" spans="1:4">
+      <c r="A8528" t="s">
+        <v>8534</v>
+      </c>
+      <c r="D8528" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8529" spans="1:4">
+      <c r="A8529" t="s">
+        <v>8535</v>
+      </c>
+      <c r="D8529" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8530" spans="1:4">
+      <c r="A8530" t="s">
+        <v>8536</v>
+      </c>
+      <c r="D8530" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8531" spans="1:4">
+      <c r="A8531" t="s">
+        <v>8537</v>
+      </c>
+      <c r="D8531" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8532" spans="1:4">
+      <c r="A8532" t="s">
+        <v>8538</v>
+      </c>
+      <c r="D8532" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8533" spans="1:4">
+      <c r="A8533" t="s">
+        <v>8539</v>
+      </c>
+      <c r="D8533" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8534" spans="1:4">
+      <c r="A8534" t="s">
+        <v>8540</v>
+      </c>
+      <c r="D8534" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8535" spans="1:4">
+      <c r="A8535" t="s">
+        <v>8541</v>
+      </c>
+      <c r="D8535" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8536" spans="1:4">
+      <c r="A8536" t="s">
+        <v>8542</v>
+      </c>
+      <c r="D8536" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8537" spans="1:4">
+      <c r="A8537" t="s">
+        <v>8543</v>
+      </c>
+      <c r="D8537" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8538" spans="1:4">
+      <c r="A8538" t="s">
+        <v>8544</v>
+      </c>
+      <c r="D8538" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8539" spans="1:4">
+      <c r="A8539" t="s">
+        <v>8545</v>
+      </c>
+      <c r="D8539" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8540" spans="1:4">
+      <c r="A8540" t="s">
+        <v>8546</v>
+      </c>
+      <c r="D8540" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8541" spans="1:4">
+      <c r="A8541" t="s">
+        <v>8547</v>
+      </c>
+      <c r="D8541" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8542" spans="1:4">
+      <c r="A8542" t="s">
+        <v>8548</v>
+      </c>
+      <c r="D8542" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>